<commit_message>
Convert catalog product names to Taiwan Traditional Chinese.
Run OpenCC s2twp during sync so DIY shelf labels and master workbook use 繁體 instead of simplified source names.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/commodity_idx.xlsx
+++ b/data/commodity_idx.xlsx
@@ -433,7 +433,7 @@
         <v>吊墜</v>
       </c>
       <c r="D2" t="str">
-        <v>丝带</v>
+        <v>絲帶</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -525,7 +525,7 @@
         <v>珍珠</v>
       </c>
       <c r="D6" t="str">
-        <v>圆珍珠</v>
+        <v>圓珍珠</v>
       </c>
       <c r="E6">
         <v>6</v>
@@ -548,7 +548,7 @@
         <v>珍珠</v>
       </c>
       <c r="D7" t="str">
-        <v>圆珍珠</v>
+        <v>圓珍珠</v>
       </c>
       <c r="E7">
         <v>8</v>
@@ -571,7 +571,7 @@
         <v>珍珠</v>
       </c>
       <c r="D8" t="str">
-        <v>圆珍珠</v>
+        <v>圓珍珠</v>
       </c>
       <c r="E8">
         <v>10</v>
@@ -594,7 +594,7 @@
         <v>隔珠</v>
       </c>
       <c r="D9" t="str">
-        <v>镂空钻蕾丝</v>
+        <v>鏤空鑽蕾絲</v>
       </c>
       <c r="E9">
         <v>6</v>
@@ -617,7 +617,7 @@
         <v>吊墜</v>
       </c>
       <c r="D10" t="str">
-        <v>满镶星星</v>
+        <v>滿鑲星星</v>
       </c>
       <c r="E10">
         <v>2</v>
@@ -640,7 +640,7 @@
         <v>吊墜</v>
       </c>
       <c r="D11" t="str">
-        <v>霹雳</v>
+        <v>霹靂</v>
       </c>
       <c r="E11">
         <v>2</v>
@@ -663,7 +663,7 @@
         <v>吊墜</v>
       </c>
       <c r="D12" t="str">
-        <v>镂空小猫</v>
+        <v>鏤空小貓</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -686,7 +686,7 @@
         <v>吊墜</v>
       </c>
       <c r="D13" t="str">
-        <v>爱心曲别针</v>
+        <v>愛心曲別針</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -709,7 +709,7 @@
         <v>隔珠</v>
       </c>
       <c r="D14" t="str">
-        <v>锆石魔盒钻</v>
+        <v>鋯石魔盒鑽</v>
       </c>
       <c r="E14">
         <v>8</v>
@@ -824,7 +824,7 @@
         <v>吊墜</v>
       </c>
       <c r="D19" t="str">
-        <v>银色满镶月亮</v>
+        <v>銀色滿鑲月亮</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -847,7 +847,7 @@
         <v>隔珠</v>
       </c>
       <c r="D20" t="str">
-        <v>锆石方钻</v>
+        <v>鋯石方鑽</v>
       </c>
       <c r="E20">
         <v>6</v>
@@ -939,7 +939,7 @@
         <v>吊墜</v>
       </c>
       <c r="D24" t="str">
-        <v>镂空金福</v>
+        <v>鏤空金福</v>
       </c>
       <c r="E24">
         <v>2</v>
@@ -1376,7 +1376,7 @@
         <v>隔珠</v>
       </c>
       <c r="D43" t="str">
-        <v>五棱银钻</v>
+        <v>五稜銀鑽</v>
       </c>
       <c r="E43">
         <v>5</v>
@@ -1399,7 +1399,7 @@
         <v>吊墜</v>
       </c>
       <c r="D44" t="str">
-        <v>锆石星星</v>
+        <v>鋯石星星</v>
       </c>
       <c r="E44">
         <v>2</v>
@@ -1422,7 +1422,7 @@
         <v>吊墜</v>
       </c>
       <c r="D45" t="str">
-        <v>寻心钥匙</v>
+        <v>尋心鑰匙</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -1445,7 +1445,7 @@
         <v>吊墜</v>
       </c>
       <c r="D46" t="str">
-        <v>白水鱼尾</v>
+        <v>白水魚尾</v>
       </c>
       <c r="E46">
         <v>2</v>
@@ -1468,7 +1468,7 @@
         <v>隔珠</v>
       </c>
       <c r="D47" t="str">
-        <v>转运柄</v>
+        <v>轉運柄</v>
       </c>
       <c r="E47">
         <v>8</v>
@@ -1491,7 +1491,7 @@
         <v>隔珠</v>
       </c>
       <c r="D48" t="str">
-        <v>恶魔之眼</v>
+        <v>惡魔之眼</v>
       </c>
       <c r="E48">
         <v>6</v>
@@ -1514,7 +1514,7 @@
         <v>隔珠</v>
       </c>
       <c r="D49" t="str">
-        <v>扭纹小环</v>
+        <v>扭紋小環</v>
       </c>
       <c r="E49">
         <v>5</v>
@@ -1537,7 +1537,7 @@
         <v>吊墜</v>
       </c>
       <c r="D50" t="str">
-        <v>星星奖章</v>
+        <v>星星獎章</v>
       </c>
       <c r="E50">
         <v>2</v>
@@ -1560,7 +1560,7 @@
         <v>隔珠</v>
       </c>
       <c r="D51" t="str">
-        <v>粉樱花</v>
+        <v>粉櫻花</v>
       </c>
       <c r="E51">
         <v>6</v>
@@ -1583,7 +1583,7 @@
         <v>隔珠</v>
       </c>
       <c r="D52" t="str">
-        <v>锆石花形钻</v>
+        <v>鋯石花形鑽</v>
       </c>
       <c r="E52">
         <v>6</v>
@@ -1675,7 +1675,7 @@
         <v>隔珠</v>
       </c>
       <c r="D56" t="str">
-        <v>锆石切割</v>
+        <v>鋯石切割</v>
       </c>
       <c r="E56">
         <v>5</v>
@@ -1698,7 +1698,7 @@
         <v>隔珠</v>
       </c>
       <c r="D57" t="str">
-        <v>交织戒</v>
+        <v>交織戒</v>
       </c>
       <c r="E57">
         <v>6</v>
@@ -1721,7 +1721,7 @@
         <v>吊墜</v>
       </c>
       <c r="D58" t="str">
-        <v>锆石晨星</v>
+        <v>鋯石晨星</v>
       </c>
       <c r="E58">
         <v>2</v>
@@ -1744,7 +1744,7 @@
         <v>隔珠</v>
       </c>
       <c r="D59" t="str">
-        <v>藏银十字架</v>
+        <v>藏銀十字架</v>
       </c>
       <c r="E59">
         <v>8</v>
@@ -1767,7 +1767,7 @@
         <v>隔珠</v>
       </c>
       <c r="D60" t="str">
-        <v>锆石切割双层</v>
+        <v>鋯石切割雙層</v>
       </c>
       <c r="E60">
         <v>6</v>
@@ -1790,7 +1790,7 @@
         <v>隔珠</v>
       </c>
       <c r="D61" t="str">
-        <v>银色小环</v>
+        <v>銀色小環</v>
       </c>
       <c r="E61">
         <v>5</v>
@@ -2020,7 +2020,7 @@
         <v>吊墜</v>
       </c>
       <c r="D71" t="str">
-        <v>满钻蝴蝶</v>
+        <v>滿鑽蝴蝶</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -2066,7 +2066,7 @@
         <v>隔珠</v>
       </c>
       <c r="D73" t="str">
-        <v>镂空金蕾丝</v>
+        <v>鏤空金蕾絲</v>
       </c>
       <c r="E73">
         <v>6</v>
@@ -2250,7 +2250,7 @@
         <v>隔珠</v>
       </c>
       <c r="D81" t="str">
-        <v>复古雕花</v>
+        <v>復古雕花</v>
       </c>
       <c r="E81">
         <v>8</v>
@@ -2342,7 +2342,7 @@
         <v>隔珠</v>
       </c>
       <c r="D85" t="str">
-        <v>小祥云</v>
+        <v>小祥雲</v>
       </c>
       <c r="E85">
         <v>5</v>
@@ -2365,7 +2365,7 @@
         <v>隔珠</v>
       </c>
       <c r="D86" t="str">
-        <v>大祥云</v>
+        <v>大祥雲</v>
       </c>
       <c r="E86">
         <v>5</v>
@@ -2595,7 +2595,7 @@
         <v>隔珠</v>
       </c>
       <c r="D96" t="str">
-        <v>锆石猫咪</v>
+        <v>鋯石貓咪</v>
       </c>
       <c r="E96">
         <v>8</v>
@@ -2687,7 +2687,7 @@
         <v>隔珠</v>
       </c>
       <c r="D100" t="str">
-        <v>五棱金钻</v>
+        <v>五稜金鑽</v>
       </c>
       <c r="E100">
         <v>5</v>
@@ -2825,7 +2825,7 @@
         <v>吊墜</v>
       </c>
       <c r="D106" t="str">
-        <v>葫芦成双</v>
+        <v>葫蘆成雙</v>
       </c>
       <c r="E106">
         <v>2</v>
@@ -2917,7 +2917,7 @@
         <v>隔珠</v>
       </c>
       <c r="D110" t="str">
-        <v>锆石螺旋</v>
+        <v>鋯石螺旋</v>
       </c>
       <c r="E110">
         <v>6</v>
@@ -2940,7 +2940,7 @@
         <v>吊墜</v>
       </c>
       <c r="D111" t="str">
-        <v>闪跃月亮</v>
+        <v>閃躍月亮</v>
       </c>
       <c r="E111">
         <v>2</v>
@@ -2963,7 +2963,7 @@
         <v>隔珠</v>
       </c>
       <c r="D112" t="str">
-        <v>锆石钻闪</v>
+        <v>鋯石鑽閃</v>
       </c>
       <c r="E112">
         <v>5</v>
@@ -2986,7 +2986,7 @@
         <v>吊墜</v>
       </c>
       <c r="D113" t="str">
-        <v>小年兽</v>
+        <v>小年獸</v>
       </c>
       <c r="E113">
         <v>2</v>
@@ -3009,7 +3009,7 @@
         <v>隔珠</v>
       </c>
       <c r="D114" t="str">
-        <v>金色小环</v>
+        <v>金色小環</v>
       </c>
       <c r="E114">
         <v>5</v>
@@ -3032,7 +3032,7 @@
         <v>吊墜</v>
       </c>
       <c r="D115" t="str">
-        <v>北极星</v>
+        <v>北極星</v>
       </c>
       <c r="E115">
         <v>2</v>
@@ -3055,7 +3055,7 @@
         <v>隔珠</v>
       </c>
       <c r="D116" t="str">
-        <v>彩锆轮</v>
+        <v>彩鋯輪</v>
       </c>
       <c r="E116">
         <v>6</v>
@@ -3147,7 +3147,7 @@
         <v>隔珠</v>
       </c>
       <c r="D120" t="str">
-        <v>醒狮</v>
+        <v>醒獅</v>
       </c>
       <c r="E120">
         <v>8</v>
@@ -3308,7 +3308,7 @@
         <v>吊墜</v>
       </c>
       <c r="D127" t="str">
-        <v>锆石彩虹</v>
+        <v>鋯石彩虹</v>
       </c>
       <c r="E127">
         <v>2</v>
@@ -3331,7 +3331,7 @@
         <v>隔珠</v>
       </c>
       <c r="D128" t="str">
-        <v>小锆石钻闪</v>
+        <v>小鋯石鑽閃</v>
       </c>
       <c r="E128">
         <v>5</v>
@@ -3515,7 +3515,7 @@
         <v>隔珠</v>
       </c>
       <c r="D136" t="str">
-        <v>银色小珠</v>
+        <v>銀色小珠</v>
       </c>
       <c r="E136">
         <v>6</v>
@@ -3607,7 +3607,7 @@
         <v>吊墜</v>
       </c>
       <c r="D140" t="str">
-        <v>金色满镶月亮</v>
+        <v>金色滿鑲月亮</v>
       </c>
       <c r="E140">
         <v>2</v>
@@ -3630,7 +3630,7 @@
         <v>隔珠</v>
       </c>
       <c r="D141" t="str">
-        <v>花边轨道</v>
+        <v>花邊軌道</v>
       </c>
       <c r="E141">
         <v>6</v>
@@ -3722,7 +3722,7 @@
         <v>隔珠</v>
       </c>
       <c r="D145" t="str">
-        <v>回财纹</v>
+        <v>回財紋</v>
       </c>
       <c r="E145">
         <v>5</v>
@@ -3745,7 +3745,7 @@
         <v>隔珠</v>
       </c>
       <c r="D146" t="str">
-        <v>藏银卷草</v>
+        <v>藏銀卷草</v>
       </c>
       <c r="E146">
         <v>6</v>
@@ -3791,7 +3791,7 @@
         <v>隔珠</v>
       </c>
       <c r="D148" t="str">
-        <v>藏银十字花</v>
+        <v>藏銀十字花</v>
       </c>
       <c r="E148">
         <v>8</v>
@@ -3883,7 +3883,7 @@
         <v>吊墜</v>
       </c>
       <c r="D152" t="str">
-        <v>藏银羽毛</v>
+        <v>藏銀羽毛</v>
       </c>
       <c r="E152">
         <v>2</v>
@@ -3975,7 +3975,7 @@
         <v>隔珠</v>
       </c>
       <c r="D156" t="str">
-        <v>藏银树叶</v>
+        <v>藏銀樹葉</v>
       </c>
       <c r="E156">
         <v>6</v>
@@ -4021,7 +4021,7 @@
         <v>隔珠</v>
       </c>
       <c r="D158" t="str">
-        <v>锆石钻闪双层</v>
+        <v>鋯石鑽閃雙層</v>
       </c>
       <c r="E158">
         <v>6</v>
@@ -4044,7 +4044,7 @@
         <v>隔珠</v>
       </c>
       <c r="D159" t="str">
-        <v>藏银瓦片</v>
+        <v>藏銀瓦片</v>
       </c>
       <c r="E159">
         <v>8</v>
@@ -4067,7 +4067,7 @@
         <v>吊墜</v>
       </c>
       <c r="D160" t="str">
-        <v>四叶草</v>
+        <v>四葉草</v>
       </c>
       <c r="E160">
         <v>2</v>
@@ -4228,7 +4228,7 @@
         <v>隔珠</v>
       </c>
       <c r="D167" t="str">
-        <v>银色六字真言</v>
+        <v>銀色六字真言</v>
       </c>
       <c r="E167">
         <v>8</v>
@@ -4251,7 +4251,7 @@
         <v>隔珠</v>
       </c>
       <c r="D168" t="str">
-        <v>凯尔特结</v>
+        <v>凱爾特結</v>
       </c>
       <c r="E168">
         <v>6</v>
@@ -4274,7 +4274,7 @@
         <v>隔珠</v>
       </c>
       <c r="D169" t="str">
-        <v>银色绣球</v>
+        <v>銀色繡球</v>
       </c>
       <c r="E169">
         <v>8</v>
@@ -4366,7 +4366,7 @@
         <v>吊墜</v>
       </c>
       <c r="D173" t="str">
-        <v>王国之泪</v>
+        <v>王國之淚</v>
       </c>
       <c r="E173">
         <v>2</v>
@@ -4964,7 +4964,7 @@
         <v>吊墜</v>
       </c>
       <c r="D199" t="str">
-        <v>藏银蝴蝶流苏</v>
+        <v>藏銀蝴蝶流蘇</v>
       </c>
       <c r="E199">
         <v>2</v>
@@ -4987,7 +4987,7 @@
         <v>隔珠</v>
       </c>
       <c r="D200" t="str">
-        <v>玫瑰花环</v>
+        <v>玫瑰花環</v>
       </c>
       <c r="E200">
         <v>6</v>
@@ -5010,7 +5010,7 @@
         <v>隔珠</v>
       </c>
       <c r="D201" t="str">
-        <v>白玛瑙魔盒</v>
+        <v>白瑪瑙魔盒</v>
       </c>
       <c r="E201">
         <v>8</v>
@@ -5033,7 +5033,7 @@
         <v>隔珠</v>
       </c>
       <c r="D202" t="str">
-        <v>藏银回纹</v>
+        <v>藏銀回紋</v>
       </c>
       <c r="E202">
         <v>5</v>
@@ -5125,7 +5125,7 @@
         <v>隔珠</v>
       </c>
       <c r="D206" t="str">
-        <v>朱砂魔盒</v>
+        <v>硃砂魔盒</v>
       </c>
       <c r="E206">
         <v>8</v>
@@ -5148,7 +5148,7 @@
         <v>吊墜</v>
       </c>
       <c r="D207" t="str">
-        <v>藏银十字吊坠</v>
+        <v>藏銀十字吊墜</v>
       </c>
       <c r="E207">
         <v>2</v>
@@ -5171,7 +5171,7 @@
         <v>吊墜</v>
       </c>
       <c r="D208" t="str">
-        <v>藏银叶丛</v>
+        <v>藏銀葉叢</v>
       </c>
       <c r="E208">
         <v>2</v>
@@ -5194,7 +5194,7 @@
         <v>隔珠</v>
       </c>
       <c r="D209" t="str">
-        <v>藏银小花立方</v>
+        <v>藏銀小花立方</v>
       </c>
       <c r="E209">
         <v>8</v>
@@ -5217,7 +5217,7 @@
         <v>隔珠</v>
       </c>
       <c r="D210" t="str">
-        <v>藏银大花立方</v>
+        <v>藏銀大花立方</v>
       </c>
       <c r="E210">
         <v>8</v>
@@ -5309,7 +5309,7 @@
         <v>隔珠</v>
       </c>
       <c r="D214" t="str">
-        <v>景泰蓝福球</v>
+        <v>景泰藍福球</v>
       </c>
       <c r="E214">
         <v>8</v>
@@ -5884,7 +5884,7 @@
         <v>吊墜</v>
       </c>
       <c r="D239" t="str">
-        <v>捕梦网</v>
+        <v>捕夢網</v>
       </c>
       <c r="E239">
         <v>2</v>

</xml_diff>

<commit_message>
Update catalog sizes and prices from new_input workbook.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/commodity_idx.xlsx
+++ b/data/commodity_idx.xlsx
@@ -564,7 +564,7 @@
         <v>8</v>
       </c>
       <c r="G6">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H6" t="str">
         <v>雪花幽灵.png</v>
@@ -593,7 +593,7 @@
         <v>10</v>
       </c>
       <c r="G7">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="H7" t="str">
         <v>雪花幽灵.png</v>
@@ -622,7 +622,7 @@
         <v>8</v>
       </c>
       <c r="G8">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H8" t="str">
         <v>白幽灵.png</v>
@@ -651,7 +651,7 @@
         <v>6</v>
       </c>
       <c r="G9">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H9" t="str">
         <v>淡水珍珠.png</v>
@@ -680,7 +680,7 @@
         <v>8</v>
       </c>
       <c r="G10">
-        <v>169</v>
+        <v>129</v>
       </c>
       <c r="H10" t="str">
         <v>淡水珍珠.png</v>
@@ -709,7 +709,7 @@
         <v>10</v>
       </c>
       <c r="G11">
-        <v>199</v>
+        <v>169</v>
       </c>
       <c r="H11" t="str">
         <v>淡水珍珠.png</v>
@@ -738,7 +738,7 @@
         <v>8</v>
       </c>
       <c r="G12">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="H12" t="str">
         <v>奶白晶.png</v>
@@ -767,7 +767,7 @@
         <v>10</v>
       </c>
       <c r="G13">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H13" t="str">
         <v>奶白晶.png</v>
@@ -851,7 +851,7 @@
         <v>2</v>
       </c>
       <c r="F16">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G16">
         <v>69</v>
@@ -880,7 +880,7 @@
         <v>5</v>
       </c>
       <c r="F17">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G17">
         <v>49</v>
@@ -909,7 +909,7 @@
         <v>2</v>
       </c>
       <c r="F18">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G18">
         <v>59</v>
@@ -970,7 +970,7 @@
         <v>8</v>
       </c>
       <c r="G20">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H20" t="str">
         <v>星光粉晶.png</v>
@@ -1115,7 +1115,7 @@
         <v>6</v>
       </c>
       <c r="G25">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="H25" t="str">
         <v>紫锂辉.png</v>
@@ -1144,7 +1144,7 @@
         <v>8</v>
       </c>
       <c r="G26">
-        <v>129</v>
+        <v>89</v>
       </c>
       <c r="H26" t="str">
         <v>紫锂辉.png</v>
@@ -1173,7 +1173,7 @@
         <v>10</v>
       </c>
       <c r="G27">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="H27" t="str">
         <v>紫锂辉.png</v>
@@ -1202,7 +1202,7 @@
         <v>8</v>
       </c>
       <c r="G28">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H28" t="str">
         <v>菱格立方.png</v>
@@ -1289,7 +1289,7 @@
         <v>10</v>
       </c>
       <c r="G31">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H31" t="str">
         <v>粉水晶.png</v>
@@ -1347,7 +1347,7 @@
         <v>14</v>
       </c>
       <c r="G33">
-        <v>599</v>
+        <v>399</v>
       </c>
       <c r="H33" t="str">
         <v>镂空金福.png</v>
@@ -1376,7 +1376,7 @@
         <v>8</v>
       </c>
       <c r="G34">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="H34" t="str">
         <v>白阿塞.png</v>
@@ -1434,7 +1434,7 @@
         <v>6</v>
       </c>
       <c r="G36">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H36" t="str">
         <v>奶油海蓝宝.png</v>
@@ -1463,7 +1463,7 @@
         <v>8</v>
       </c>
       <c r="G37">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H37" t="str">
         <v>奶油海蓝宝.png</v>
@@ -1492,7 +1492,7 @@
         <v>10</v>
       </c>
       <c r="G38">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="H38" t="str">
         <v>奶油海蓝宝.png</v>
@@ -1579,7 +1579,7 @@
         <v>6</v>
       </c>
       <c r="G41">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H41" t="str">
         <v>海纹石.png</v>
@@ -1608,7 +1608,7 @@
         <v>8</v>
       </c>
       <c r="G42">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H42" t="str">
         <v>海纹石.png</v>
@@ -1637,7 +1637,7 @@
         <v>10</v>
       </c>
       <c r="G43">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="H43" t="str">
         <v>海纹石.png</v>
@@ -1695,7 +1695,7 @@
         <v>8</v>
       </c>
       <c r="G45">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H45" t="str">
         <v>金发晶.png</v>
@@ -1724,7 +1724,7 @@
         <v>10</v>
       </c>
       <c r="G46">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H46" t="str">
         <v>金发晶.png</v>
@@ -1753,7 +1753,7 @@
         <v>14</v>
       </c>
       <c r="G47">
-        <v>699</v>
+        <v>499</v>
       </c>
       <c r="H47" t="str">
         <v>白水鱼尾.png</v>
@@ -1782,7 +1782,7 @@
         <v>10</v>
       </c>
       <c r="G48">
-        <v>399</v>
+        <v>299</v>
       </c>
       <c r="H48" t="str">
         <v>转运柄.png</v>
@@ -1898,7 +1898,7 @@
         <v>8</v>
       </c>
       <c r="G52">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="H52" t="str">
         <v>薰衣草.png</v>
@@ -1950,13 +1950,13 @@
         <v>粉櫻花</v>
       </c>
       <c r="E54">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F54">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G54">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H54" t="str">
         <v>粉樱花.png</v>
@@ -1985,7 +1985,7 @@
         <v>10</v>
       </c>
       <c r="G55">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H55" t="str">
         <v>锆石花形钻.png</v>
@@ -2072,7 +2072,7 @@
         <v>8</v>
       </c>
       <c r="G58">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H58" t="str">
         <v>黄水晶.png</v>
@@ -2101,7 +2101,7 @@
         <v>10</v>
       </c>
       <c r="G59">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H59" t="str">
         <v>黄水晶.png</v>
@@ -2188,7 +2188,7 @@
         <v>7</v>
       </c>
       <c r="G62">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H62" t="str">
         <v>钛钢4.png</v>
@@ -2275,7 +2275,7 @@
         <v>7</v>
       </c>
       <c r="G65">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H65" t="str">
         <v>钛钢9.png</v>
@@ -2304,7 +2304,7 @@
         <v>6</v>
       </c>
       <c r="G66">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H66" t="str">
         <v>桂花.png</v>
@@ -2420,7 +2420,7 @@
         <v>6</v>
       </c>
       <c r="G70">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H70" t="str">
         <v>蜜蜡.png</v>
@@ -2449,7 +2449,7 @@
         <v>8</v>
       </c>
       <c r="G71">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H71" t="str">
         <v>蜜蜡.png</v>
@@ -2478,7 +2478,7 @@
         <v>10</v>
       </c>
       <c r="G72">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H72" t="str">
         <v>银饰R.png</v>
@@ -2536,7 +2536,7 @@
         <v>7</v>
       </c>
       <c r="G74">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H74" t="str">
         <v>钛钢7.png</v>
@@ -2623,7 +2623,7 @@
         <v>7</v>
       </c>
       <c r="G77">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H77" t="str">
         <v>钛钢0.png</v>
@@ -2681,7 +2681,7 @@
         <v>10</v>
       </c>
       <c r="G79">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H79" t="str">
         <v>银饰J.png</v>
@@ -2710,7 +2710,7 @@
         <v>7</v>
       </c>
       <c r="G80">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H80" t="str">
         <v>钛钢6.png</v>
@@ -2797,7 +2797,7 @@
         <v>10</v>
       </c>
       <c r="G83">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H83" t="str">
         <v>银饰I.png</v>
@@ -2826,7 +2826,7 @@
         <v>10</v>
       </c>
       <c r="G84">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H84" t="str">
         <v>银饰U.png</v>
@@ -2855,7 +2855,7 @@
         <v>7</v>
       </c>
       <c r="G85">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H85" t="str">
         <v>钛钢3.png</v>
@@ -2884,7 +2884,7 @@
         <v>7</v>
       </c>
       <c r="G86">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H86" t="str">
         <v>钛钢2.png</v>
@@ -2913,7 +2913,7 @@
         <v>7</v>
       </c>
       <c r="G87">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H87" t="str">
         <v>钛钢8.png</v>
@@ -2942,7 +2942,7 @@
         <v>7</v>
       </c>
       <c r="G88">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H88" t="str">
         <v>钛钢5.png</v>
@@ -3000,7 +3000,7 @@
         <v>10</v>
       </c>
       <c r="G90">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H90" t="str">
         <v>银饰P.png</v>
@@ -3058,7 +3058,7 @@
         <v>8</v>
       </c>
       <c r="G92">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H92" t="str">
         <v>绿发晶.png</v>
@@ -3116,7 +3116,7 @@
         <v>10</v>
       </c>
       <c r="G94">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H94" t="str">
         <v>银饰C.png</v>
@@ -3145,7 +3145,7 @@
         <v>10</v>
       </c>
       <c r="G95">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H95" t="str">
         <v>银饰B.png</v>
@@ -3203,7 +3203,7 @@
         <v>10</v>
       </c>
       <c r="G97">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H97" t="str">
         <v>银饰O.png</v>
@@ -3232,7 +3232,7 @@
         <v>10</v>
       </c>
       <c r="G98">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H98" t="str">
         <v>银饰W.png</v>
@@ -3258,7 +3258,7 @@
         <v>2</v>
       </c>
       <c r="F99">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G99">
         <v>59</v>
@@ -3319,7 +3319,7 @@
         <v>10</v>
       </c>
       <c r="G101">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H101" t="str">
         <v>银饰Q.png</v>
@@ -3348,7 +3348,7 @@
         <v>10</v>
       </c>
       <c r="G102">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="H102" t="str">
         <v>羽毛萤石.png</v>
@@ -3406,7 +3406,7 @@
         <v>10</v>
       </c>
       <c r="G104">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H104" t="str">
         <v>银饰F.png</v>
@@ -3461,7 +3461,7 @@
         <v>3</v>
       </c>
       <c r="F106">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="G106">
         <v>299</v>
@@ -3522,7 +3522,7 @@
         <v>10</v>
       </c>
       <c r="G108">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H108" t="str">
         <v>银饰N.png</v>
@@ -3551,7 +3551,7 @@
         <v>10</v>
       </c>
       <c r="G109">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H109" t="str">
         <v>银饰M.png</v>
@@ -3580,7 +3580,7 @@
         <v>10</v>
       </c>
       <c r="G110">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H110" t="str">
         <v>银饰H.png</v>
@@ -3638,7 +3638,7 @@
         <v>10</v>
       </c>
       <c r="G112">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H112" t="str">
         <v>银饰G.png</v>
@@ -3696,7 +3696,7 @@
         <v>10</v>
       </c>
       <c r="G114">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H114" t="str">
         <v>银饰T.png</v>
@@ -3725,7 +3725,7 @@
         <v>10</v>
       </c>
       <c r="G115">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H115" t="str">
         <v>银饰E.png</v>
@@ -3754,7 +3754,7 @@
         <v>10</v>
       </c>
       <c r="G116">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H116" t="str">
         <v>银饰K.png</v>
@@ -3812,7 +3812,7 @@
         <v>10</v>
       </c>
       <c r="G118">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H118" t="str">
         <v>银饰V.png</v>
@@ -3870,7 +3870,7 @@
         <v>10</v>
       </c>
       <c r="G120">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H120" t="str">
         <v>银饰L.png</v>
@@ -3899,7 +3899,7 @@
         <v>10</v>
       </c>
       <c r="G121">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H121" t="str">
         <v>银饰A.png</v>
@@ -3957,7 +3957,7 @@
         <v>10</v>
       </c>
       <c r="G123">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H123" t="str">
         <v>银饰Y.png</v>
@@ -4073,7 +4073,7 @@
         <v>10</v>
       </c>
       <c r="G127">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H127" t="str">
         <v>银饰X.png</v>
@@ -4160,7 +4160,7 @@
         <v>10</v>
       </c>
       <c r="G130">
-        <v>199</v>
+        <v>169</v>
       </c>
       <c r="H130" t="str">
         <v>琥珀石.png</v>
@@ -4247,7 +4247,7 @@
         <v>10</v>
       </c>
       <c r="G133">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H133" t="str">
         <v>银饰Z.png</v>
@@ -4363,7 +4363,7 @@
         <v>10</v>
       </c>
       <c r="G137">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H137" t="str">
         <v>银饰D.png</v>
@@ -4450,7 +4450,7 @@
         <v>10</v>
       </c>
       <c r="G140">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="H140" t="str">
         <v>海蓝宝.png</v>
@@ -4479,7 +4479,7 @@
         <v>10</v>
       </c>
       <c r="G141">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="H141" t="str">
         <v>银饰S.png</v>
@@ -4566,7 +4566,7 @@
         <v>6</v>
       </c>
       <c r="G144">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="H144" t="str">
         <v>黄塔晶.png</v>
@@ -4595,7 +4595,7 @@
         <v>8</v>
       </c>
       <c r="G145">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="H145" t="str">
         <v>黄塔晶.png</v>
@@ -4624,7 +4624,7 @@
         <v>10</v>
       </c>
       <c r="G146">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="H146" t="str">
         <v>黄塔晶.png</v>
@@ -4711,7 +4711,7 @@
         <v>8</v>
       </c>
       <c r="G149">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H149" t="str">
         <v>黑发晶.png</v>
@@ -4769,7 +4769,7 @@
         <v>7</v>
       </c>
       <c r="G151">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H151" t="str">
         <v>天珠.png</v>
@@ -4798,7 +4798,7 @@
         <v>4</v>
       </c>
       <c r="G152">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H152" t="str">
         <v>银色小珠.png</v>
@@ -5143,10 +5143,10 @@
         <v>2</v>
       </c>
       <c r="F164">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="G164">
-        <v>599</v>
+        <v>399</v>
       </c>
       <c r="H164" t="str">
         <v>藏银羽毛.png</v>
@@ -5175,7 +5175,7 @@
         <v>6</v>
       </c>
       <c r="G165">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H165" t="str">
         <v>绿萤石.png</v>
@@ -5204,7 +5204,7 @@
         <v>8</v>
       </c>
       <c r="G166">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H166" t="str">
         <v>绿萤石.png</v>
@@ -5262,7 +5262,7 @@
         <v>8</v>
       </c>
       <c r="G168">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H168" t="str">
         <v>蔷薇石.png</v>
@@ -5291,7 +5291,7 @@
         <v>10</v>
       </c>
       <c r="G169">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H169" t="str">
         <v>蔷薇石.png</v>
@@ -5320,7 +5320,7 @@
         <v>4</v>
       </c>
       <c r="G170">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H170" t="str">
         <v>金色小珠.png</v>
@@ -5407,7 +5407,7 @@
         <v>7</v>
       </c>
       <c r="G173">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="H173" t="str">
         <v>锆石钻闪双层.png</v>
@@ -5523,7 +5523,7 @@
         <v>6</v>
       </c>
       <c r="G177">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H177" t="str">
         <v>月光石.png</v>
@@ -5639,7 +5639,7 @@
         <v>8</v>
       </c>
       <c r="G181">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H181" t="str">
         <v>太阳石.png</v>
@@ -5668,7 +5668,7 @@
         <v>10</v>
       </c>
       <c r="G182">
-        <v>169</v>
+        <v>129</v>
       </c>
       <c r="H182" t="str">
         <v>太阳石.png</v>
@@ -5726,7 +5726,7 @@
         <v>10</v>
       </c>
       <c r="G184">
-        <v>699</v>
+        <v>599</v>
       </c>
       <c r="H184" t="str">
         <v>圣海蓝宝.png</v>
@@ -5871,7 +5871,7 @@
         <v>6</v>
       </c>
       <c r="G189">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H189" t="str">
         <v>紫水晶.png</v>
@@ -5929,7 +5929,7 @@
         <v>10</v>
       </c>
       <c r="G191">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H191" t="str">
         <v>紫水晶.png</v>
@@ -5955,10 +5955,10 @@
         <v>2</v>
       </c>
       <c r="F192">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G192">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H192" t="str">
         <v>国王之泪.png</v>
@@ -6103,7 +6103,7 @@
         <v>8</v>
       </c>
       <c r="G197">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H197" t="str">
         <v>紫粉晶.png</v>
@@ -6132,7 +6132,7 @@
         <v>10</v>
       </c>
       <c r="G198">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H198" t="str">
         <v>紫粉晶.png</v>
@@ -6219,7 +6219,7 @@
         <v>6</v>
       </c>
       <c r="G201">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="H201" t="str">
         <v>草莓晶.png</v>
@@ -6248,7 +6248,7 @@
         <v>8</v>
       </c>
       <c r="G202">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H202" t="str">
         <v>草莓晶.png</v>
@@ -6277,7 +6277,7 @@
         <v>10</v>
       </c>
       <c r="G203">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H203" t="str">
         <v>草莓晶.png</v>
@@ -6332,10 +6332,10 @@
         <v>2</v>
       </c>
       <c r="F205">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="G205">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H205" t="str">
         <v>藏银蝴蝶流苏.png</v>
@@ -6393,7 +6393,7 @@
         <v>8</v>
       </c>
       <c r="G207">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H207" t="str">
         <v>藏银十字.png</v>
@@ -6451,7 +6451,7 @@
         <v>11</v>
       </c>
       <c r="G209">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H209" t="str">
         <v>景泰蓝.png</v>
@@ -6509,7 +6509,7 @@
         <v>8</v>
       </c>
       <c r="G211">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H211" t="str">
         <v>黑金超.png</v>
@@ -6538,7 +6538,7 @@
         <v>10</v>
       </c>
       <c r="G212">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H212" t="str">
         <v>黑金超.png</v>
@@ -6857,7 +6857,7 @@
         <v>8</v>
       </c>
       <c r="G223">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H223" t="str">
         <v>银曜石.png</v>
@@ -6886,7 +6886,7 @@
         <v>10</v>
       </c>
       <c r="G224">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H224" t="str">
         <v>银曜石.png</v>
@@ -6912,7 +6912,7 @@
         <v>2</v>
       </c>
       <c r="F225">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G225">
         <v>69</v>
@@ -6944,7 +6944,7 @@
         <v>6</v>
       </c>
       <c r="G226">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="H226" t="str">
         <v>朱砂.png</v>
@@ -6973,7 +6973,7 @@
         <v>6</v>
       </c>
       <c r="G227">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H227" t="str">
         <v>蓝晶石.png</v>
@@ -7031,7 +7031,7 @@
         <v>10</v>
       </c>
       <c r="G229">
-        <v>199</v>
+        <v>169</v>
       </c>
       <c r="H229" t="str">
         <v>蓝晶石.png</v>
@@ -7234,7 +7234,7 @@
         <v>6</v>
       </c>
       <c r="G236">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H236" t="str">
         <v>孔雀石.png</v>
@@ -7292,7 +7292,7 @@
         <v>10</v>
       </c>
       <c r="G238">
-        <v>199</v>
+        <v>169</v>
       </c>
       <c r="H238" t="str">
         <v>孔雀石.png</v>
@@ -7321,7 +7321,7 @@
         <v>6</v>
       </c>
       <c r="G239">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H239" t="str">
         <v>青金石.png</v>
@@ -7408,7 +7408,7 @@
         <v>6</v>
       </c>
       <c r="G242">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H242" t="str">
         <v>乌拉圭.png</v>
@@ -7437,7 +7437,7 @@
         <v>8</v>
       </c>
       <c r="G243">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H243" t="str">
         <v>乌拉圭.png</v>
@@ -7466,7 +7466,7 @@
         <v>10</v>
       </c>
       <c r="G244">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="H244" t="str">
         <v>乌拉圭.png</v>
@@ -7495,7 +7495,7 @@
         <v>6</v>
       </c>
       <c r="G245">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="H245" t="str">
         <v>紫幽灵.png</v>
@@ -7640,7 +7640,7 @@
         <v>6</v>
       </c>
       <c r="G250">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H250" t="str">
         <v>紫金砂.png</v>
@@ -7669,7 +7669,7 @@
         <v>8</v>
       </c>
       <c r="G251">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H251" t="str">
         <v>紫金砂.png</v>
@@ -7698,7 +7698,7 @@
         <v>10</v>
       </c>
       <c r="G252">
-        <v>129</v>
+        <v>99</v>
       </c>
       <c r="H252" t="str">
         <v>紫金砂.png</v>
@@ -7756,7 +7756,7 @@
         <v>8</v>
       </c>
       <c r="G254">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H254" t="str">
         <v>金曜石.png</v>
@@ -7785,7 +7785,7 @@
         <v>10</v>
       </c>
       <c r="G255">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H255" t="str">
         <v>金曜石.png</v>
@@ -7843,7 +7843,7 @@
         <v>8</v>
       </c>
       <c r="G257">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H257" t="str">
         <v>黑曜石.png</v>
@@ -7872,7 +7872,7 @@
         <v>10</v>
       </c>
       <c r="G258">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H258" t="str">
         <v>黑曜石.png</v>

</xml_diff>

<commit_message>
Add 聖藍方糖 and 青金石跑環 to catalog and Shopify import.
Keep newly dropped lifestyle *1.* images during catalog sync so long-press photos are not deleted before mapping.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/commodity_idx.xlsx
+++ b/data/commodity_idx.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I258"/>
+  <dimension ref="A1:I260"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7216,36 +7216,36 @@
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>kqs_stn_6</v>
+        <v>slft_ft_8</v>
       </c>
       <c r="B236" t="str">
-        <v>珠子</v>
+        <v>配件</v>
       </c>
       <c r="C236" t="str">
-        <v>礦石</v>
+        <v>方糖</v>
       </c>
       <c r="D236" t="str">
-        <v>孔雀石</v>
+        <v>聖藍方糖</v>
       </c>
       <c r="E236">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F236">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G236">
         <v>59</v>
       </c>
       <c r="H236" t="str">
-        <v>孔雀石.png</v>
+        <v>圣蓝方糖.png</v>
       </c>
       <c r="I236" t="str">
-        <v/>
+        <v>龍海市上全</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>kqs_stn_8</v>
+        <v>kqs_stn_6</v>
       </c>
       <c r="B237" t="str">
         <v>珠子</v>
@@ -7257,13 +7257,13 @@
         <v>孔雀石</v>
       </c>
       <c r="E237">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F237">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G237">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="H237" t="str">
         <v>孔雀石.png</v>
@@ -7274,7 +7274,7 @@
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>kqs_stn_10</v>
+        <v>kqs_stn_8</v>
       </c>
       <c r="B238" t="str">
         <v>珠子</v>
@@ -7286,13 +7286,13 @@
         <v>孔雀石</v>
       </c>
       <c r="E238">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F238">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G238">
-        <v>169</v>
+        <v>89</v>
       </c>
       <c r="H238" t="str">
         <v>孔雀石.png</v>
@@ -7303,7 +7303,7 @@
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>qjs_stn_6</v>
+        <v>kqs_stn_10</v>
       </c>
       <c r="B239" t="str">
         <v>珠子</v>
@@ -7312,19 +7312,19 @@
         <v>礦石</v>
       </c>
       <c r="D239" t="str">
-        <v>青金石</v>
+        <v>孔雀石</v>
       </c>
       <c r="E239">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F239">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G239">
-        <v>59</v>
+        <v>169</v>
       </c>
       <c r="H239" t="str">
-        <v>青金石.png</v>
+        <v>孔雀石.png</v>
       </c>
       <c r="I239" t="str">
         <v/>
@@ -7332,7 +7332,7 @@
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>qjs_stn_8</v>
+        <v>qjs_stn_6</v>
       </c>
       <c r="B240" t="str">
         <v>珠子</v>
@@ -7344,13 +7344,13 @@
         <v>青金石</v>
       </c>
       <c r="E240">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F240">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G240">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="H240" t="str">
         <v>青金石.png</v>
@@ -7361,7 +7361,7 @@
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>qjs_stn_10</v>
+        <v>qjs_stn_8</v>
       </c>
       <c r="B241" t="str">
         <v>珠子</v>
@@ -7373,13 +7373,13 @@
         <v>青金石</v>
       </c>
       <c r="E241">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F241">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G241">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H241" t="str">
         <v>青金石.png</v>
@@ -7390,28 +7390,28 @@
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>wlg_cysl_6</v>
+        <v>qjs_stn_10</v>
       </c>
       <c r="B242" t="str">
         <v>珠子</v>
       </c>
       <c r="C242" t="str">
-        <v>水晶</v>
+        <v>礦石</v>
       </c>
       <c r="D242" t="str">
-        <v>烏拉圭</v>
+        <v>青金石</v>
       </c>
       <c r="E242">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F242">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G242">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="H242" t="str">
-        <v>乌拉圭.png</v>
+        <v>青金石.png</v>
       </c>
       <c r="I242" t="str">
         <v/>
@@ -7419,7 +7419,7 @@
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>wlg_cysl_8</v>
+        <v>wlg_cysl_6</v>
       </c>
       <c r="B243" t="str">
         <v>珠子</v>
@@ -7431,13 +7431,13 @@
         <v>烏拉圭</v>
       </c>
       <c r="E243">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F243">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G243">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="H243" t="str">
         <v>乌拉圭.png</v>
@@ -7448,7 +7448,7 @@
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>wlg_cysl_10</v>
+        <v>wlg_cysl_8</v>
       </c>
       <c r="B244" t="str">
         <v>珠子</v>
@@ -7460,13 +7460,13 @@
         <v>烏拉圭</v>
       </c>
       <c r="E244">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F244">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G244">
-        <v>159</v>
+        <v>89</v>
       </c>
       <c r="H244" t="str">
         <v>乌拉圭.png</v>
@@ -7477,7 +7477,7 @@
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>zyl_cysl_6</v>
+        <v>wlg_cysl_10</v>
       </c>
       <c r="B245" t="str">
         <v>珠子</v>
@@ -7486,19 +7486,19 @@
         <v>水晶</v>
       </c>
       <c r="D245" t="str">
-        <v>紫幽靈</v>
+        <v>烏拉圭</v>
       </c>
       <c r="E245">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F245">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G245">
-        <v>49</v>
+        <v>159</v>
       </c>
       <c r="H245" t="str">
-        <v>紫幽灵.png</v>
+        <v>乌拉圭.png</v>
       </c>
       <c r="I245" t="str">
         <v/>
@@ -7506,45 +7506,45 @@
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>zyl_cysl_8</v>
+        <v>qjsph_ph_4</v>
       </c>
       <c r="B246" t="str">
-        <v>珠子</v>
+        <v>配件</v>
       </c>
       <c r="C246" t="str">
-        <v>水晶</v>
+        <v>跑環</v>
       </c>
       <c r="D246" t="str">
-        <v>紫幽靈</v>
+        <v>青金石跑環</v>
       </c>
       <c r="E246">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F246">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G246">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="H246" t="str">
-        <v>紫幽灵.png</v>
+        <v>青金石跑环.png</v>
       </c>
       <c r="I246" t="str">
-        <v/>
+        <v>義烏晶德</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>he_agt_6</v>
+        <v>zyl_cysl_6</v>
       </c>
       <c r="B247" t="str">
         <v>珠子</v>
       </c>
       <c r="C247" t="str">
-        <v>瑪瑙</v>
+        <v>水晶</v>
       </c>
       <c r="D247" t="str">
-        <v>黑瑪瑙</v>
+        <v>紫幽靈</v>
       </c>
       <c r="E247">
         <v>6</v>
@@ -7553,10 +7553,10 @@
         <v>6</v>
       </c>
       <c r="G247">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="H247" t="str">
-        <v>黑玛瑙.png</v>
+        <v>紫幽灵.png</v>
       </c>
       <c r="I247" t="str">
         <v/>
@@ -7564,16 +7564,16 @@
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>he_agt_8</v>
+        <v>zyl_cysl_8</v>
       </c>
       <c r="B248" t="str">
         <v>珠子</v>
       </c>
       <c r="C248" t="str">
-        <v>瑪瑙</v>
+        <v>水晶</v>
       </c>
       <c r="D248" t="str">
-        <v>黑瑪瑙</v>
+        <v>紫幽靈</v>
       </c>
       <c r="E248">
         <v>8</v>
@@ -7585,7 +7585,7 @@
         <v>59</v>
       </c>
       <c r="H248" t="str">
-        <v>黑玛瑙.png</v>
+        <v>紫幽灵.png</v>
       </c>
       <c r="I248" t="str">
         <v/>
@@ -7593,7 +7593,7 @@
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>he_agt_10</v>
+        <v>he_agt_6</v>
       </c>
       <c r="B249" t="str">
         <v>珠子</v>
@@ -7605,13 +7605,13 @@
         <v>黑瑪瑙</v>
       </c>
       <c r="E249">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F249">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G249">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="H249" t="str">
         <v>黑玛瑙.png</v>
@@ -7622,28 +7622,28 @@
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>zjs_stn_6</v>
+        <v>he_agt_8</v>
       </c>
       <c r="B250" t="str">
         <v>珠子</v>
       </c>
       <c r="C250" t="str">
-        <v>礦石</v>
+        <v>瑪瑙</v>
       </c>
       <c r="D250" t="str">
-        <v>紫金砂</v>
+        <v>黑瑪瑙</v>
       </c>
       <c r="E250">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F250">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G250">
         <v>59</v>
       </c>
       <c r="H250" t="str">
-        <v>紫金砂.png</v>
+        <v>黑玛瑙.png</v>
       </c>
       <c r="I250" t="str">
         <v/>
@@ -7651,28 +7651,28 @@
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>zjs_stn_8</v>
+        <v>he_agt_10</v>
       </c>
       <c r="B251" t="str">
         <v>珠子</v>
       </c>
       <c r="C251" t="str">
-        <v>礦石</v>
+        <v>瑪瑙</v>
       </c>
       <c r="D251" t="str">
-        <v>紫金砂</v>
+        <v>黑瑪瑙</v>
       </c>
       <c r="E251">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F251">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G251">
         <v>89</v>
       </c>
       <c r="H251" t="str">
-        <v>紫金砂.png</v>
+        <v>黑玛瑙.png</v>
       </c>
       <c r="I251" t="str">
         <v/>
@@ -7680,7 +7680,7 @@
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>zjs_stn_10</v>
+        <v>zjs_stn_6</v>
       </c>
       <c r="B252" t="str">
         <v>珠子</v>
@@ -7692,13 +7692,13 @@
         <v>紫金砂</v>
       </c>
       <c r="E252">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F252">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G252">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="H252" t="str">
         <v>紫金砂.png</v>
@@ -7709,7 +7709,7 @@
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>jys_stn_6</v>
+        <v>zjs_stn_8</v>
       </c>
       <c r="B253" t="str">
         <v>珠子</v>
@@ -7718,19 +7718,19 @@
         <v>礦石</v>
       </c>
       <c r="D253" t="str">
-        <v>金曜石</v>
+        <v>紫金砂</v>
       </c>
       <c r="E253">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F253">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G253">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="H253" t="str">
-        <v>金曜石.png</v>
+        <v>紫金砂.png</v>
       </c>
       <c r="I253" t="str">
         <v/>
@@ -7738,7 +7738,7 @@
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>jys_stn_8</v>
+        <v>zjs_stn_10</v>
       </c>
       <c r="B254" t="str">
         <v>珠子</v>
@@ -7747,19 +7747,19 @@
         <v>礦石</v>
       </c>
       <c r="D254" t="str">
-        <v>金曜石</v>
+        <v>紫金砂</v>
       </c>
       <c r="E254">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F254">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G254">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="H254" t="str">
-        <v>金曜石.png</v>
+        <v>紫金砂.png</v>
       </c>
       <c r="I254" t="str">
         <v/>
@@ -7767,7 +7767,7 @@
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>jys_stn_10</v>
+        <v>jys_stn_6</v>
       </c>
       <c r="B255" t="str">
         <v>珠子</v>
@@ -7779,13 +7779,13 @@
         <v>金曜石</v>
       </c>
       <c r="E255">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F255">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G255">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="H255" t="str">
         <v>金曜石.png</v>
@@ -7796,7 +7796,7 @@
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>hys_stn_6</v>
+        <v>jys_stn_8</v>
       </c>
       <c r="B256" t="str">
         <v>珠子</v>
@@ -7805,19 +7805,19 @@
         <v>礦石</v>
       </c>
       <c r="D256" t="str">
-        <v>黑曜石</v>
+        <v>金曜石</v>
       </c>
       <c r="E256">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F256">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G256">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="H256" t="str">
-        <v>黑曜石.png</v>
+        <v>金曜石.png</v>
       </c>
       <c r="I256" t="str">
         <v/>
@@ -7825,7 +7825,7 @@
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>hys_stn_8</v>
+        <v>jys_stn_10</v>
       </c>
       <c r="B257" t="str">
         <v>珠子</v>
@@ -7834,19 +7834,19 @@
         <v>礦石</v>
       </c>
       <c r="D257" t="str">
-        <v>黑曜石</v>
+        <v>金曜石</v>
       </c>
       <c r="E257">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F257">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G257">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="H257" t="str">
-        <v>黑曜石.png</v>
+        <v>金曜石.png</v>
       </c>
       <c r="I257" t="str">
         <v/>
@@ -7854,7 +7854,7 @@
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>hys_stn_10</v>
+        <v>hys_stn_6</v>
       </c>
       <c r="B258" t="str">
         <v>珠子</v>
@@ -7866,13 +7866,13 @@
         <v>黑曜石</v>
       </c>
       <c r="E258">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F258">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G258">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="H258" t="str">
         <v>黑曜石.png</v>
@@ -7881,9 +7881,67 @@
         <v/>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>hys_stn_8</v>
+      </c>
+      <c r="B259" t="str">
+        <v>珠子</v>
+      </c>
+      <c r="C259" t="str">
+        <v>礦石</v>
+      </c>
+      <c r="D259" t="str">
+        <v>黑曜石</v>
+      </c>
+      <c r="E259">
+        <v>8</v>
+      </c>
+      <c r="F259">
+        <v>8</v>
+      </c>
+      <c r="G259">
+        <v>59</v>
+      </c>
+      <c r="H259" t="str">
+        <v>黑曜石.png</v>
+      </c>
+      <c r="I259" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>hys_stn_10</v>
+      </c>
+      <c r="B260" t="str">
+        <v>珠子</v>
+      </c>
+      <c r="C260" t="str">
+        <v>礦石</v>
+      </c>
+      <c r="D260" t="str">
+        <v>黑曜石</v>
+      </c>
+      <c r="E260">
+        <v>10</v>
+      </c>
+      <c r="F260">
+        <v>10</v>
+      </c>
+      <c r="G260">
+        <v>89</v>
+      </c>
+      <c r="H260" t="str">
+        <v>黑曜石.png</v>
+      </c>
+      <c r="I260" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I258"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I260"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>